<commit_message>
Gemisch: neue Verdichtung (90 bar, dicht kuehlen) in Skript und Excel
- excel_werte_gemisch.py: p_V = 90 bar (Cricondenbar 82,2 + 3 bar Unsicherheit,
  Reserve), Kuehlen auf 20 degC in der dichten Phase statt Verfluessigen im
  Zweiphasengebiet; alte Verdichtung (60 bar wie reines CO2) zum Vergleich;
  Diagrammdaten bis 120 degC
- 04: Mappe zeigt neue Kette (1 Stufe > 95 degC, 2 Stufen Pflicht, Kuehler,
  Pumpe auf 114,9 bar), alte Verdichtung als Pfad im Phasendiagramm und als
  Vergleichsblock auf "Gemisch & Grenzen"
- 03: rechnet ueber excel_werte_gemisch.werte() - gleiche Zahlen wie die Mappe,
  Diagramme mit alter und neuer Verdichtung

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FLRXDCKem3dbasHw8H8HkL
</commit_message>
<xml_diff>
--- a/Masterarbeit/Einspeicherung/Begleitstoffe_CO2/CO2_Zwischenspeicher_Rechenuebersicht_Gemisch.xlsx
+++ b/Masterarbeit/Einspeicherung/Begleitstoffe_CO2/CO2_Zwischenspeicher_Rechenuebersicht_Gemisch.xlsx
@@ -139,7 +139,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1115" uniqueCount="615">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1161" uniqueCount="661">
   <si>
     <t>CO₂-Zwischenspeicherung in Salzkavernen – Obertageanlage</t>
   </si>
@@ -1497,18 +1497,24 @@
   <si>
     <t xml:space="preserve">Diese Mappe zeigt Schritt für Schritt, wie die Obertageanlage für die Einspeicherung berechnet wird:
 1. Welcher Druck muss am Bohrlochkopf anliegen? → das gibt die Kaverne über die Gassäule vor.
-2. Wie bringt die Anlage das CO₂ auf diesen Druck? → Pumpe (dichte Anlieferung, S1) bzw. Verdichter, Verflüssiger und Pumpe (gasförmige Anlieferung, S2).
+2. Wie bringt die Anlage das CO₂ auf diesen Druck? → Pumpe (dichte Anlieferung, S1) bzw. Verdichter, Kühler und Pumpe (gasförmige Anlieferung, S2).
 3. Wo liegen alle Zustände im Phasendiagramm – und wo liegt das Betriebsfenster von Bohrloch und Kaverne?
 Diese Mappe rechnet das Worst-Case-Gemisch mit 5 % Begleitstoffen – gleicher Aufbau wie die Mappe für reines CO₂. Was sich an den Grenzen ändert und warum: Blatt „Gemisch &amp; Grenzen“.</t>
   </si>
   <si>
+    <t xml:space="preserve">Anlieferung gasförmig: Verdichtung (2 Stufen), Zwischenkühlung, Kühlung in der dichten Phase, Pumpe.</t>
+  </si>
+  <si>
     <t xml:space="preserve">→ Gemisch &amp; Grenzen</t>
   </si>
   <si>
     <t xml:space="preserve">Was die Begleitstoffe ändern: Zweiphasengebiet, Unsicherheit ±3 bar, neue Grenzen der Anlage.</t>
   </si>
   <si>
-    <t xml:space="preserve">Gemisch: Blasendruck bei T_K = 76,7 bar + 3 bar Unsicherheit → sicher flüssig (reines CO₂: 60 bar)</t>
+    <t xml:space="preserve">Enddruck Verdichtung = Kühlerdruck</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gemisch: ≥ Cricondenbar 82,2 + 3 bar → Kühlen ohne Zweiphasengebiet (rein: 60 bar, verflüssigen)</t>
   </si>
   <si>
     <t xml:space="preserve">Gemisch: ≤ Taudruck(T_K) − 3 bar = 60,4 bar; Stufe 2 ≤ 95 °C ab 48,1 bar → zulässig ca. 48–60 bar</t>
@@ -1520,13 +1526,13 @@
     <t xml:space="preserve">S2 Basisfall 1 Stufe: spezifische Arbeit gesamt</t>
   </si>
   <si>
-    <t xml:space="preserve">Verdichter + Pumpe; 1 Stufe erreicht 100,3 °C &gt; 95 °C (Q-016)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pflicht beim Gemisch (1 Stufe &gt; 95 °C); spart außerdem rund 10%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S2 braucht rund 10% weniger Arbeit – deshalb verflüssigen und pumpen</t>
+    <t xml:space="preserve">Verdichter + Pumpe; 1 Stufe erreicht 111,6 °C &gt; 95 °C (Q-016)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pflicht beim Gemisch (1 Stufe &gt; 95 °C); spart außerdem rund 13%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S2 (2 Stufen) braucht rund 14% weniger Arbeit – deshalb dicht kühlen und pumpen</t>
   </si>
   <si>
     <t xml:space="preserve">Einspeicherung, Kaverne V1 (tief) · Stillstand: Temperatur = Gebirgstemperatur · Worst-Case-Gemisch</t>
@@ -1595,46 +1601,73 @@
     <t xml:space="preserve">dicht (flüssig)</t>
   </si>
   <si>
-    <t xml:space="preserve">Einspeicherung S2 – gasförmige Anlieferung: verdichten, verflüssigen, pumpen (Worst-Case-Gemisch)</t>
+    <t xml:space="preserve">Einspeicherung S2 – gasförmige Anlieferung: verdichten, dicht kühlen, pumpen (Worst-Case-Gemisch)</t>
   </si>
   <si>
     <t xml:space="preserve">AUSGANGSLAGE:  Das CO₂-Gemisch kommt gasförmig an: 30 bar, 15 °C (Annahme).
 Q-016:  Bielka, Kuczyński, Nagy (2023): CO₂ Compression and Dehydration for Transport and Geological Storage. Energies 16, 1804 (AGH Krakau). Übersichtsarbeit zu Abscheidung, Trocknung, Transport und Speicherstandortwahl – plus eine eigene Prozesssimulation (BR&amp;E ProMax, Peng-Robinson): CO₂ aus einer Rauchgasabscheidung (1,51 bar, 35 °C, 2,45 Mio. t/a ≈ 78 kg/s) wird in 5 Stufen auf 100 bar verdichtet, mit TEG getrocknet und auf 20 °C gekühlt – flüssig für den Pipelinetransport zu einer Speicherstätte in 30 km Entfernung (S. 5: 74 bar sind das Minimum, üblich 100 bar als Reserve für Druckverluste).
 Annahmen aus Q 16 (S. 4, Kap. 2.3):  Kühlung auf 20 °C nach jeder Stufe · höchstens 95 °C nach jeder Stufe · Wirkungsgrad 84 % in Stufe 1, je weitere Stufe −2 % · zum Schluss Kühlung auf 20 °C → flüssig. Q-016 verdichtet für die Pipeline, hier für den Bohrlochkopf – das Druckniveau (100 bzw. 114,9 bar) und der Massenstrom (78 bzw. 27–54 kg/s) sind vergleichbar. NICHT übernommen: 45 bar Zwischendruck (für die TEG-Trocknung gewählt, Glykol schließt OGE aus).
-VERFLÜSSIGEN BEIM GEMISCH:  Die Begleitstoffe heben den Druck, ab dem bei 20 °C alles flüssig ist, von 57,3 bar (Dampfdruck reines CO₂) auf 76,7 bar (Blasendruck). Mit 3 bar Unsicherheit der Phasengrenze → p_V = 80 bar. Die Kondensation läuft über einen Temperaturgleit: sie beginnt bei 80 bar bei 27,9 °C (Taulinie) und ist bei 23,7 °C (Blasenlinie) abgeschlossen.
-ZAHL DER STUFEN:  Beim Gemisch reicht eine Stufe NICHT mehr: bis 80 bar erreicht sie 100,3 °C und überschreitet die 95-°C-Grenze aus Q-016 (reines CO₂ bis 60 bar: 73,2 °C). Die zweistufige Variante unten ist deshalb Pflicht – sie spart außerdem 10% Arbeit.
-RECHENWEG:  Verdichter und Pumpe wie in S1: isentrop + Wirkungsgrad, h_aus = h_ein + (h_s − h_ein) / η. Verflüssiger: abgeführte Wärme je kg q = h_vor − h_nach.
-GRENZEN:  20 °C setzen Kühlwasser voraus. Mit Luftkühlung (ca. 35 °C) läge die Kühltemperatur über der kritischen Temperatur des Gemischs (28,0 °C) – dann gäbe es keine Kondensation mehr.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Blasendruck bei T_K (Gemisch)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CoolProp: p(Q = 0, T_K)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Abstand p_V − p_Blase</t>
-  </si>
-  <si>
-    <t xml:space="preserve">muss ≥ 3 bar sein (Unsicherheit der Phasengrenze)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Blasentemperatur bei p_V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CoolProp: T(Q = 0, p_V) – Kondensation beginnt bei 27,9 °C</t>
-  </si>
-  <si>
-    <t xml:space="preserve">flüssig</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S2 braucht rund 18-mal so viel Arbeit wie S1 – und rund 10% weniger als Durchverdichten. Beim Gemisch ist die zweite Verdichterstufe Pflicht (1 Stufe: 100,3 °C &gt; 95 °C) und spart weitere 10%.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AUFBAU:  Stufe 1 30 → 49,0 bar, Zwischenkühlung auf 20 °C (das Gemisch bleibt gasförmig: Taudruck bei 20 °C = 63,4 bar), Stufe 2 → 80 bar. Zwischendruck mit gleichem Druckverhältnis in beiden Stufen: p_zw = √(p_ein · p_V). Wirkungsgrade 84 / 82 % (Q-016). Verflüssiger und Pumpe wie im Basisfall. Beim Gemisch ist diese Variante Pflicht (95-°C-Grenze).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FRAGE:  Warum nicht einfach gasförmig bis 114,9 bar durchverdichten, statt zu verflüssigen und zu pumpen?
+NEUE VERDICHTUNG BEIM GEMISCH:  Reines CO₂ wird bei 60 bar und 20 °C verflüssigt (Dampfdruck 57,3 bar). Das Gemisch hat bei 20 °C ein Zweiphasengebiet von 63,4 bar (Taulinie) bis 76,7 bar (Blasenlinie) – bei 60 bar bliebe es gasförmig (alte Verdichtung, Blatt „Gemisch &amp; Grenzen“). Deshalb wird über die Cricondenbar (82,2 bar = höchster Druck des Zweiphasengebiets) + 3 bar Unsicherheit verdichtet: p_V = 90 bar. Dort kühlt der Kühler von der Verdichteraustrittstemperatur auf 20 °C, ohne das Zweiphasengebiet zu berühren – das Gemisch geht stetig in die dichte Phase über, es wird nichts kondensiert (wie Q-016: Endstufe 100 bar, dann 20 °C). Danach bringt die Pumpe das dichte Gemisch auf 114,9 bar.
+ZAHL DER STUFEN:  Eine Stufe bis 90 bar erreicht 111,6 °C und überschreitet die 95-°C-Grenze aus Q-016 (reines CO₂ bis 60 bar: 73,2 °C). Die zweistufige Variante unten ist deshalb Pflicht – sie spart außerdem 13% Arbeit.
+RECHENWEG:  Verdichter und Pumpe wie in S1: isentrop + Wirkungsgrad, h_aus = h_ein + (h_s − h_ein) / η. Kühler: abgeführte Wärme je kg q = h_vor − h_nach.
+GRENZEN:  20 °C setzen Kühlwasser voraus. Mit Luftkühlung (ca. 35 °C) läge die Kühltemperatur über der kritischen Temperatur des Gemischs (28,0 °C): das Gemisch wäre dann vor der Pumpe überkritisch und deutlich weniger dicht.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Netzübergabe → Messtechnik/Filtration → Verdichter → Kühler (dicht) → Pumpe → Bohrlochkopf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kühler (dichte Phase)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Austrittsdruck = Kühlerdruck p_V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cricondenbar Gemisch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CoolProp: höchster Druck der Phasengrenze</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Abstand p_V − Cricondenbar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">muss ≥ 3 bar sein, dann kein Zweiphasengebiet beim Kühlen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blasendruck bei T_K</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CoolProp: p(Q = 0, T_K) – Taudruck 63,4 bar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enthalpie nach Kühler</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phase nach Kühler</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dicht (flüssig)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kühlleistung Kühler, oberer Fall</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S2 (2 Stufen) braucht rund 17-mal so viel Arbeit wie S1 – und rund 14% weniger als Durchverdichten. Beim Gemisch ist die zweite Verdichterstufe Pflicht (1 Stufe: 111,6 °C &gt; 95 °C) und spart gegenüber einer Stufe 13%.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUFBAU:  Stufe 1 30 → 52,0 bar, Zwischenkühlung auf 20 °C (das Gemisch bleibt gasförmig: Taudruck bei 20 °C = 63,4 bar), Stufe 2 → 90 bar. Zwischendruck mit gleichem Druckverhältnis in beiden Stufen: p_zw = √(p_ein · p_V). Wirkungsgrade 84 / 82 % (Q-016). Kühler und Pumpe wie im Basisfall. Beim Gemisch ist diese Variante Pflicht (95-°C-Grenze).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Variante: zweistufige Verdichtung bis zum Kühlerdruck p_V (sonst wie Basisfall)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kühler und Pumpe wie Basisfall</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Abgeführte Wärme Kühler</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FRAGE:  Warum nicht einfach gasförmig bis 114,9 bar durchverdichten, statt dicht zu kühlen und zu pumpen?
 AUFBAU nach denselben Regeln aus Q-016:  Zwischenkühlung auf 20 °C, höchstens 95 °C je Stufe, Wirkungsgrade 84 / 82 %. Der Zwischendruck muss mit 3 bar Abstand unter dem Taudruck des Gemischs bei 20 °C bleiben (63,4 − 3 = 60,4 bar; reines CO₂: 57,3 bar), sonst beginnt die Kondensation schon im Zwischenkühler; und die zweite Stufe darf 95 °C nicht überschreiten (ab 48,1 bar). Daraus folgt ein zulässiger Bereich von ca. 48–60 bar – gewählt wie bei reinem CO₂ 50 bar.
 FAIRER VERGLEICH:  Am Ende kühlt ein Nachkühler auf denselben Endzustand wie S2 (gleicher Druck, gleiche Temperatur).</t>
   </si>
@@ -1642,7 +1675,10 @@
     <t xml:space="preserve">p_zw ≤ p_Tau(T_K) − 3 bar ?</t>
   </si>
   <si>
-    <t xml:space="preserve">S2 Basisfall: 1 Stufe (&gt; 95 °C!) + Verflüssiger + Pumpe</t>
+    <t xml:space="preserve">S2 Basisfall: 1 Stufe (&gt; 95 °C!) + Kühler + Pumpe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S2 Variante: 2 Stufen + Kühler + Pumpe</t>
   </si>
   <si>
     <t xml:space="preserve">Phasendiagramm – Prozesspfade der Einspeicherung und Betriebsfenster von Bohrloch und Kaverne (Worst-Case-Gemisch)</t>
@@ -1651,7 +1687,7 @@
     <t xml:space="preserve">Worst-Case-Gemisch (95 % CO₂ + 5 % Begleitstoffe) · Stoffdaten CoolProp (GERG-2008-Mischungsregel) · Fest-Gebiet, Sublimations- und Schmelzlinie: Näherung reines CO₂ (Span &amp; Wagner 1996)</t>
   </si>
   <si>
-    <t xml:space="preserve">DIAGRAMM 1:  Farbflächen = Phasengebiete des Gemischs, rot = Zweiphasengebiet (reines CO₂ hat nur eine Linie, grau zum Vergleich). Rot gestrichelt = ±3 bar Unsicherheit der Phasengrenze. Grün = S1 (Pumpe). Blau = S2 Basisfall (1 Stufe bis 80 bar, 100,3 °C &gt; 95 °C). Hellblau gepunktet = S2-Variante mit 2 Stufen (beim Gemisch Pflicht). Violett gestrichelt = Durchverdichten (2 Stufen bis 114,9 bar, dann Nachkühler).
+    <t xml:space="preserve">DIAGRAMM 1:  Farbflächen = Phasengebiete des Gemischs, rot = Zweiphasengebiet (reines CO₂ hat nur eine Linie, grau zum Vergleich). Rot gestrichelt = ±3 bar Unsicherheit der Phasengrenze. Grün = S1 (Pumpe). Blau = S2 Basisfall (1 Stufe bis 90 bar, 111,6 °C &gt; 95 °C, Kühler dicht auf 20 °C, Pumpe). Grau gestrichelt = alte Verdichtung wie reines CO₂ (60 bar) – bleibt beim Gemisch gasförmig, die Pumpe könnte nicht fördern. Hellblau gepunktet = S2-Variante mit 2 Stufen (beim Gemisch Pflicht). Violett gestrichelt = Durchverdichten (2 Stufen bis 114,9 bar, dann Nachkühler).
 ENDPUNKT:  Alle Pfade enden am Bohrlochkopf bei 114,9 bar (reines CO₂: 107,6 bar). Diagramm 2 zeigt Bohrloch und Kaverne – nur im Stillstand.</t>
   </si>
   <si>
@@ -1659,7 +1695,7 @@
 BETRIEBSFENSTER IM STILLSTAND:  Der Bereich zwischen der Linie „voll“ (oben) und der Linie „leer“ (unten), links begrenzt durch den Kopf-Balken und rechts durch den Kavernen-Balken.
 WICHTIG BEI LEERER KAVERNE:  70 bar unten ergeben oben 50,7 bar (reines CO₂: 45,0 bar). Das obere Bohrloch (0–82 m) liegt dann im Zweiphasengebiet des Gemischs. Erst ab ca. 171,2 bar Kavernendruck (Grenzfall: Kopf = Cricondenbar 82,2 bar) bleibt das ganze Bohrloch einphasig.
 KAVERNE SELBST:  Bei 46 °C liegt sie immer über der Cricondentherm des Gemischs (28,1 °C) – dort gibt es keine Flüssigphase. Über 81,5 bar ist das Gemisch überkritisch, bei 70 bar gasförmig.
-STILLSTAND VS. BETRIEB:  Die Gassäulen sind mit Gebirgstemperatur gerechnet (Kopf 10 °C) und gelten nur, solange nichts fließt. Beim Einspeichern kommt das Gemisch wärmer aus der Pumpe (S1 18,4 °C, S2 27,0 °C).</t>
+STILLSTAND VS. BETRIEB:  Die Gassäulen sind mit Gebirgstemperatur gerechnet (Kopf 10 °C) und gelten nur, solange nichts fließt. Beim Einspeichern kommt das Gemisch wärmer aus der Pumpe (S1 18,4 °C, S2 24,4 °C).</t>
   </si>
   <si>
     <t xml:space="preserve">—</t>
@@ -1710,6 +1746,9 @@
     <t xml:space="preserve">Kritischer Punkt Gemisch</t>
   </si>
   <si>
+    <t xml:space="preserve">S2: verdichten → dicht kühlen → pumpen</t>
+  </si>
+  <si>
     <t xml:space="preserve">Gassäule Grenzfall (Kopf = Cricondenbar)</t>
   </si>
   <si>
@@ -1725,6 +1764,9 @@
     <t xml:space="preserve">Taulinie − 3 bar (sicher gasförmig)</t>
   </si>
   <si>
+    <t xml:space="preserve">Alte Verdichtung (60 bar wie reines CO₂) – bleibt gasförmig</t>
+  </si>
+  <si>
     <t xml:space="preserve">Gemisch &amp; Grenzen – was die Begleitstoffe am Phasendiagramm ändern</t>
   </si>
   <si>
@@ -1923,16 +1965,16 @@
     <t xml:space="preserve">Einspeicherung S1</t>
   </si>
   <si>
-    <t xml:space="preserve">Verflüssigungsdruck bei 20 °C</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&gt; 57,3 bar (gewählt 60)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">≥ 79,7 bar (gewählt 80)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Verflüssiger bei 80 statt 60 bar; Kondensation über Temperaturgleit 27,9 → 23,7 °C</t>
+    <t xml:space="preserve">Enddruck Verdichtung = Kühlerdruck bei 20 °C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&gt; 57,3 bar (gewählt 60, verflüssigen)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">≥ 85,2 bar (gewählt 90)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">über der Cricondenbar kühlen: kein Zweiphasengebiet, Gemisch wird stetig dicht</t>
   </si>
   <si>
     <t xml:space="preserve">Einspeicherung S2</t>
@@ -1944,7 +1986,7 @@
     <t xml:space="preserve">73,2 °C ✔</t>
   </si>
   <si>
-    <t xml:space="preserve">100,3 °C ✘ (&gt; 95 °C)</t>
+    <t xml:space="preserve">111,6 °C ✘ (&gt; 95 °C)</t>
   </si>
   <si>
     <t xml:space="preserve">zwei Verdichterstufen mit Zwischenkühlung nötig</t>
@@ -2022,7 +2064,7 @@
     <t xml:space="preserve">28,0 °C</t>
   </si>
   <si>
-    <t xml:space="preserve">Kühlung muss unter 28 °C liegen, sonst keine Kondensation (Luftkühlung reicht nicht)</t>
+    <t xml:space="preserve">Kühlung unter 28 °C nötig, sonst ist das Gemisch vor der Pumpe überkritisch</t>
   </si>
   <si>
     <t xml:space="preserve">Einspeicherung S2</t>
@@ -2037,10 +2079,106 @@
     <t xml:space="preserve">756,0 kg/m³</t>
   </si>
   <si>
-    <t xml:space="preserve">-7.5 % Masse je m³ Kavernenvolumen</t>
+    <t xml:space="preserve">-7,5 % Masse je m³ Kavernenvolumen</t>
   </si>
   <si>
     <t xml:space="preserve">Kaverne &amp; Gassäule</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alte und neue Verdichtung (S2, gasförmige Anlieferung 30 bar / 15 °C)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">alte Verdichtung (wie reines CO₂)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">neue Verdichtung (Gemisch)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Warum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enddruck Verdichtung = Druck beim Kühlen auf 20 °C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">60 bar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">90 bar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cricondenbar 82,2 bar + 3 bar Unsicherheit = 85,2 bar Minimum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verdichterstufen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 Stufe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 Stufen (Zwischenkühlung auf 20 °C)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 Stufe bis 90 bar: 111,6 °C &gt; 95 °C (Q-016)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Austrittstemperatur Verdichter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">73,7 °C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">60,9 / 65,2 °C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">höchstens 95 °C je Stufe (Q-016)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zwischendruck</t>
+  </si>
+  <si>
+    <t xml:space="preserve">–</t>
+  </si>
+  <si>
+    <t xml:space="preserve">52,0 bar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gasförmig: ≤ Taudruck(20 °C) − 3 = 60,4 bar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zustand nach Kühlung auf 20 °C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gasförmig ✘</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dicht (flüssig) ✔</t>
+  </si>
+  <si>
+    <t xml:space="preserve">alt: 3,4 bar unter der Taulinie (63,4 bar) – nichts kondensiert, die Pumpe kann Gas nicht fördern; neu: 7,8 bar über der Cricondenbar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spezifische Arbeit Verdichter + Pumpe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">– (Kette funktioniert nicht)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">62,8 kJ/kg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">reines CO₂ (alt, 1 Stufe): 46,4 kJ/kg; Durchverdichten Gemisch: 72,9 kJ/kg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Druck am Bohrlochkopf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">–</t>
+  </si>
+  <si>
+    <t xml:space="preserve">114,9 bar (Pumpe, 24,4 °C)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">wird mit der neuen Kette erreicht</t>
   </si>
 </sst>
 </file>
@@ -6377,10 +6515,10 @@
                   <c:v>S1 dichte Phase - Pumpe</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>S2 Basisfall: 1 Stufe + Verflüssiger + Pumpe</c:v>
+                  <c:v>S2 Basisfall: 1 Stufe (&gt; 95 °C!) + Kühler + Pumpe</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>S2 Variante: 2 Stufen + Verflüssiger + Pumpe</c:v>
+                  <c:v>S2 Variante: 2 Stufen + Kühler + Pumpe</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>Vergleich: Durchverdichten</c:v>
@@ -6476,10 +6614,10 @@
                   <c:v>S1 dichte Phase - Pumpe</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>S2 Basisfall: 1 Stufe + Verflüssiger + Pumpe</c:v>
+                  <c:v>S2 Basisfall: 1 Stufe (&gt; 95 °C!) + Kühler + Pumpe</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>S2 Variante: 2 Stufen + Verflüssiger + Pumpe</c:v>
+                  <c:v>S2 Variante: 2 Stufen + Kühler + Pumpe</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>Vergleich: Durchverdichten</c:v>
@@ -6575,10 +6713,10 @@
                   <c:v>S1 dichte Phase - Pumpe</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>S2 Basisfall: 1 Stufe + Verflüssiger + Pumpe</c:v>
+                  <c:v>S2 Basisfall: 1 Stufe (&gt; 95 °C!) + Kühler + Pumpe</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>S2 Variante: 2 Stufen + Verflüssiger + Pumpe</c:v>
+                  <c:v>S2 Variante: 2 Stufen + Kühler + Pumpe</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>Vergleich: Durchverdichten</c:v>
@@ -6770,12 +6908,12 @@
           </c:spPr>
           <c:cat>
             <c:strRef>
-              <c:f>Diagrammdaten!$C$8:$C$388</c:f>
+              <c:f>Diagrammdaten!$C$8:$C$408</c:f>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Diagrammdaten!$D$8:$D$388</c:f>
+              <c:f>Diagrammdaten!$D$8:$D$408</c:f>
             </c:numRef>
           </c:val>
           <c:extLst>
@@ -6802,12 +6940,12 @@
           </c:spPr>
           <c:cat>
             <c:strRef>
-              <c:f>Diagrammdaten!$C$8:$C$388</c:f>
+              <c:f>Diagrammdaten!$C$8:$C$408</c:f>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Diagrammdaten!$H$8:$H$388</c:f>
+              <c:f>Diagrammdaten!$H$8:$H$408</c:f>
             </c:numRef>
           </c:val>
           <c:extLst>
@@ -6834,17 +6972,17 @@
           </c:spPr>
           <c:cat>
             <c:strRef>
-              <c:f>Diagrammdaten!$C$8:$C$388</c:f>
+              <c:f>Diagrammdaten!$C$8:$C$408</c:f>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Diagrammdaten!$E$8:$E$388</c:f>
+              <c:f>Diagrammdaten!$E$8:$E$408</c:f>
             </c:numRef>
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{EB9F7967-7233-42AC-883E-375511FD2ED5}"/>
+              <c16:uniqueId val="{28D07E07-C023-4ECD-870E-13AA6C8CDC2F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6866,12 +7004,12 @@
           </c:spPr>
           <c:cat>
             <c:strRef>
-              <c:f>Diagrammdaten!$C$8:$C$388</c:f>
+              <c:f>Diagrammdaten!$C$8:$C$408</c:f>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Diagrammdaten!$F$8:$F$388</c:f>
+              <c:f>Diagrammdaten!$F$8:$F$408</c:f>
             </c:numRef>
           </c:val>
           <c:extLst>
@@ -6898,12 +7036,12 @@
           </c:spPr>
           <c:cat>
             <c:strRef>
-              <c:f>Diagrammdaten!$C$8:$C$388</c:f>
+              <c:f>Diagrammdaten!$C$8:$C$408</c:f>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Diagrammdaten!$G$8:$G$388</c:f>
+              <c:f>Diagrammdaten!$G$8:$G$408</c:f>
             </c:numRef>
           </c:val>
           <c:extLst>
@@ -6989,7 +7127,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{7EA1B671-CCC0-4C57-8A59-2801D70BFB76}"/>
+              <c16:uniqueId val="{28AF6CD0-FAB6-4B46-BECB-E6C9786AEB10}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -7024,7 +7162,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{B924F44C-0CB6-4B97-AA84-F40707F40138}"/>
+              <c16:uniqueId val="{0C5DAFDC-93B1-4C2A-B555-8642D3222335}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -7059,13 +7197,48 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{67BD0CDD-E244-45B9-9C95-B9540A77C2B4}"/>
+              <c16:uniqueId val="{27F775D9-02B9-4371-BD1B-712FA633E212}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="9"/>
           <c:order val="9"/>
+          <c:tx>
+            <c:v>Alte Verdichtung (60 bar wie reines CO₂) – bleibt gasförmig</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="22225" cap="rnd">
+              <a:solidFill>
+                <a:srgbClr val="7F7F7F"/>
+              </a:solidFill>
+              <a:prstDash val="sysDash"/>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Diagrammdaten!$L$360:$L$362</c:f>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Diagrammdaten!$K$360:$K$362</c:f>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{6C0AA2A5-6154-4E3E-8BCA-DD82C8EBAE85}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="10"/>
+          <c:order val="10"/>
           <c:tx>
             <c:v>Sublimationslinie</c:v>
           </c:tx>
@@ -7097,8 +7270,8 @@
           </c:extLst>
         </c:ser>
         <c:ser>
-          <c:idx val="10"/>
-          <c:order val="10"/>
+          <c:idx val="11"/>
+          <c:order val="11"/>
           <c:tx>
             <c:v>Schmelzlinie</c:v>
           </c:tx>
@@ -7130,8 +7303,8 @@
           </c:extLst>
         </c:ser>
         <c:ser>
-          <c:idx val="11"/>
-          <c:order val="11"/>
+          <c:idx val="12"/>
+          <c:order val="12"/>
           <c:tx>
             <c:v>Tripelpunkt</c:v>
           </c:tx>
@@ -7172,8 +7345,8 @@
           </c:extLst>
         </c:ser>
         <c:ser>
-          <c:idx val="12"/>
-          <c:order val="12"/>
+          <c:idx val="13"/>
+          <c:order val="13"/>
           <c:tx>
             <c:v>Kritischer Punkt Gemisch</c:v>
           </c:tx>
@@ -7214,8 +7387,8 @@
           </c:extLst>
         </c:ser>
         <c:ser>
-          <c:idx val="13"/>
-          <c:order val="13"/>
+          <c:idx val="14"/>
+          <c:order val="14"/>
           <c:tx>
             <c:v>S1: Pumpe</c:v>
           </c:tx>
@@ -7258,10 +7431,10 @@
           </c:extLst>
         </c:ser>
         <c:ser>
-          <c:idx val="14"/>
-          <c:order val="14"/>
+          <c:idx val="15"/>
+          <c:order val="15"/>
           <c:tx>
-            <c:v>S2: verdichten → verflüssigen → pumpen</c:v>
+            <c:v>S2: verdichten → dicht kühlen → pumpen</c:v>
           </c:tx>
           <c:spPr>
             <a:ln w="28575">
@@ -7302,8 +7475,8 @@
           </c:extLst>
         </c:ser>
         <c:ser>
-          <c:idx val="15"/>
-          <c:order val="15"/>
+          <c:idx val="16"/>
+          <c:order val="16"/>
           <c:tx>
             <c:v>S2-Variante: 2 Verdichterstufen</c:v>
           </c:tx>
@@ -7347,8 +7520,8 @@
           </c:extLst>
         </c:ser>
         <c:ser>
-          <c:idx val="16"/>
-          <c:order val="16"/>
+          <c:idx val="17"/>
+          <c:order val="17"/>
           <c:tx>
             <c:v>Vergleich: Durchverdichten (2 Stufen)</c:v>
           </c:tx>
@@ -7392,8 +7565,8 @@
           </c:extLst>
         </c:ser>
         <c:ser>
-          <c:idx val="17"/>
-          <c:order val="17"/>
+          <c:idx val="18"/>
+          <c:order val="18"/>
           <c:tx>
             <c:v>Beschriftung Phasengebiete E</c:v>
           </c:tx>
@@ -7572,7 +7745,7 @@
                   <c15:showDataLabelsRange val="0"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                  <c16:uniqueId val="{F1C76B3A-1B70-4E0D-97B2-B0AE772C0073}"/>
+                  <c16:uniqueId val="{B750E01B-0F4A-4249-B032-5F9874652826}"/>
                 </c:ext>
               </c:extLst>
             </c:dLbl>
@@ -7615,8 +7788,8 @@
           </c:extLst>
         </c:ser>
         <c:ser>
-          <c:idx val="18"/>
-          <c:order val="18"/>
+          <c:idx val="19"/>
+          <c:order val="19"/>
           <c:tx>
             <c:v>Beschriftung Punkte E</c:v>
           </c:tx>
@@ -7744,7 +7917,7 @@
                           <a:srgbClr val="404040"/>
                         </a:solidFill>
                       </a:rPr>
-                      <a:t>Verflüssiger</a:t>
+                      <a:t>Kühler (dicht)</a:t>
                     </a:r>
                   </a:p>
                 </c:rich>
@@ -8111,11 +8284,11 @@
         <c:delete val="1"/>
       </c:legendEntry>
       <c:legendEntry>
-        <c:idx val="17"/>
+        <c:idx val="18"/>
         <c:delete val="1"/>
       </c:legendEntry>
       <c:legendEntry>
-        <c:idx val="18"/>
+        <c:idx val="19"/>
         <c:delete val="1"/>
       </c:legendEntry>
       <c:overlay val="0"/>
@@ -8213,12 +8386,12 @@
           </c:spPr>
           <c:cat>
             <c:strRef>
-              <c:f>Diagrammdaten!$C$8:$C$388</c:f>
+              <c:f>Diagrammdaten!$C$8:$C$408</c:f>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Diagrammdaten!$D$8:$D$388</c:f>
+              <c:f>Diagrammdaten!$D$8:$D$408</c:f>
             </c:numRef>
           </c:val>
           <c:extLst>
@@ -8245,12 +8418,12 @@
           </c:spPr>
           <c:cat>
             <c:strRef>
-              <c:f>Diagrammdaten!$C$8:$C$388</c:f>
+              <c:f>Diagrammdaten!$C$8:$C$408</c:f>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Diagrammdaten!$H$8:$H$388</c:f>
+              <c:f>Diagrammdaten!$H$8:$H$408</c:f>
             </c:numRef>
           </c:val>
           <c:extLst>
@@ -8277,17 +8450,17 @@
           </c:spPr>
           <c:cat>
             <c:strRef>
-              <c:f>Diagrammdaten!$C$8:$C$388</c:f>
+              <c:f>Diagrammdaten!$C$8:$C$408</c:f>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Diagrammdaten!$E$8:$E$388</c:f>
+              <c:f>Diagrammdaten!$E$8:$E$408</c:f>
             </c:numRef>
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{79AE4295-7AA2-446F-9E0B-6019E9C6F8C5}"/>
+              <c16:uniqueId val="{7C35CBBB-6EA3-44B2-BC38-A5AE65D0D8B3}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -8309,12 +8482,12 @@
           </c:spPr>
           <c:cat>
             <c:strRef>
-              <c:f>Diagrammdaten!$C$8:$C$388</c:f>
+              <c:f>Diagrammdaten!$C$8:$C$408</c:f>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Diagrammdaten!$F$8:$F$388</c:f>
+              <c:f>Diagrammdaten!$F$8:$F$408</c:f>
             </c:numRef>
           </c:val>
           <c:extLst>
@@ -8341,12 +8514,12 @@
           </c:spPr>
           <c:cat>
             <c:strRef>
-              <c:f>Diagrammdaten!$C$8:$C$388</c:f>
+              <c:f>Diagrammdaten!$C$8:$C$408</c:f>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Diagrammdaten!$G$8:$G$388</c:f>
+              <c:f>Diagrammdaten!$G$8:$G$408</c:f>
             </c:numRef>
           </c:val>
           <c:extLst>
@@ -8432,7 +8605,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{84E97742-3EE4-4656-8FC2-740CA744D32C}"/>
+              <c16:uniqueId val="{CF5447D6-510F-4E14-9218-3637217E5DE1}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -8467,7 +8640,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{1929A488-D642-46C3-A9D5-2416841400B5}"/>
+              <c16:uniqueId val="{E5C45836-B4EE-42A6-8E56-20130147B2CD}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -8502,7 +8675,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{0ECC6D3D-3E6E-4A80-9290-6EF6839D0822}"/>
+              <c16:uniqueId val="{96F5D590-65C8-41FF-ADFD-7436542838A0}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -9005,7 +9178,7 @@
                   <c15:showDataLabelsRange val="0"/>
                 </c:ext>
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                  <c16:uniqueId val="{D96A9CE3-31E3-4490-BF49-CA180C41C4AD}"/>
+                  <c16:uniqueId val="{554A1EEB-B63E-4FCA-AD27-06D33811F8A4}"/>
                 </c:ext>
               </c:extLst>
             </c:dLbl>
@@ -10732,7 +10905,7 @@
               <a:latin typeface="Calibri"/>
               <a:cs typeface="Calibri"/>
             </a:rPr>
-            <a:t>Verflüssiger</a:t>
+            <a:t>Kühler (dicht)</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -12004,7 +12177,7 @@
               <a:latin typeface="Calibri"/>
               <a:cs typeface="Calibri"/>
             </a:rPr>
-            <a:t>→ 80 bar · 61 °C (2 Stufen)</a:t>
+            <a:t>→ 90 bar · 65 °C (2 Stufen)</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -12074,7 +12247,7 @@
               <a:latin typeface="Calibri"/>
               <a:cs typeface="Calibri"/>
             </a:rPr>
-            <a:t>80 bar · 20 °C</a:t>
+            <a:t>90 bar · 20 °C (dicht)</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -12144,7 +12317,7 @@
               <a:latin typeface="Calibri"/>
               <a:cs typeface="Calibri"/>
             </a:rPr>
-            <a:t>→ 114,9 bar · 27,0 °C</a:t>
+            <a:t>→ 114,9 bar · 24,4 °C</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -13895,7 +14068,7 @@
       <c r="C16" s="34"/>
       <c r="D16" s="34"/>
       <c r="E16" s="35" t="s">
-        <v>20</v>
+        <v>443</v>
       </c>
       <c r="F16" s="35"/>
       <c r="G16" s="35"/>
@@ -13970,10 +14143,10 @@
     </row>
     <row r="20">
       <c r="B20" s="34" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="E20" s="35" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
     </row>
     <row r="21" spans="2:15" ht="15.75" x14ac:dyDescent="0.25">
@@ -14309,7 +14482,7 @@
     </row>
     <row r="50" spans="2:15" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B50" s="33" t="s">
-        <v>57</v>
+        <v>446</v>
       </c>
       <c r="C50" s="33"/>
       <c r="D50" s="33"/>
@@ -14317,20 +14490,20 @@
         <v>58</v>
       </c>
       <c r="F50" s="4">
-        <v>80.0</v>
+        <v>90.0</v>
       </c>
       <c r="G50" s="13" t="s">
         <v>40</v>
       </c>
       <c r="H50" s="33" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="I50" s="33"/>
       <c r="J50" s="33"/>
       <c r="K50" s="33"/>
       <c r="L50" s="33"/>
       <c r="M50" s="5">
-        <v>80.0</v>
+        <v>90.0</v>
       </c>
       <c r="N50" s="33" t="str">
         <f t="shared" si="0"/>
@@ -14354,7 +14527,7 @@
         <v>40</v>
       </c>
       <c r="H51" s="33" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="I51" s="33"/>
       <c r="J51" s="33"/>
@@ -14979,7 +15152,7 @@
         <v>40</v>
       </c>
       <c r="H76" s="33" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="I76" s="33"/>
       <c r="J76" s="33"/>
@@ -15072,7 +15245,7 @@
     </row>
     <row r="80" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B80" s="33" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="C80" s="33"/>
       <c r="D80" s="33"/>
@@ -15081,13 +15254,13 @@
       </c>
       <c r="F80" s="21">
         <f>Szen2_w_ges</f>
-        <v>65.5471831342539</v>
+        <v>71.7517958185455</v>
       </c>
       <c r="G80" s="13" t="s">
         <v>128</v>
       </c>
       <c r="H80" s="33" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="I80" s="33"/>
       <c r="J80" s="33"/>
@@ -15108,7 +15281,7 @@
       </c>
       <c r="F81" s="22">
         <f>Szen2_Pmax</f>
-        <v>3521.85925064942</v>
+        <v>3855.23395165087</v>
       </c>
       <c r="G81" s="13" t="s">
         <v>131</v>
@@ -15135,13 +15308,13 @@
       </c>
       <c r="F82" s="21">
         <f>Szen2v_w_ges</f>
-        <v>58.9488615175487</v>
+        <v>62.7706612823467</v>
       </c>
       <c r="G82" s="13" t="s">
         <v>128</v>
       </c>
       <c r="H82" s="33" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="I82" s="33"/>
       <c r="J82" s="33"/>
@@ -15168,7 +15341,7 @@
         <v>128</v>
       </c>
       <c r="H83" s="33" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="I83" s="33"/>
       <c r="J83" s="33"/>
@@ -15420,7 +15593,7 @@
     </row>
     <row r="2" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B2" s="2" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
     </row>
     <row r="3" spans="2:10" x14ac:dyDescent="0.25">
@@ -15430,7 +15603,7 @@
     </row>
     <row r="4" spans="2:10" ht="117.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="32" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="C4" s="32"/>
       <c r="D4" s="32"/>
@@ -15629,7 +15802,7 @@
         <v>89.0171361957802</v>
       </c>
       <c r="I19" s="33" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="J19" s="33"/>
       <c r="K19" s="33"/>
@@ -15658,7 +15831,7 @@
         <v>19.2945413272735</v>
       </c>
       <c r="I20" s="33" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="J20" s="33"/>
       <c r="K20" s="33"/>
@@ -16366,7 +16539,7 @@
     </row>
     <row r="74" spans="2:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B74" s="36" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="C74" s="36"/>
       <c r="D74" s="36"/>
@@ -16454,7 +16627,7 @@
     </row>
     <row r="4" spans="2:8" ht="77.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="32" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="C4" s="32"/>
       <c r="D4" s="32"/>
@@ -16473,7 +16646,7 @@
         <v>185</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="D7" s="12" t="s">
         <v>187</v>
@@ -16595,7 +16768,7 @@
     </row>
     <row r="14" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B14" s="25" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
     </row>
     <row r="16" spans="2:8" x14ac:dyDescent="0.25">
@@ -16625,7 +16798,7 @@
     </row>
     <row r="18" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B18" s="10" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="C18" s="5">
         <v>114.93130198208927</v>
@@ -16641,7 +16814,7 @@
         <v>755.9538427162327</v>
       </c>
       <c r="G18" s="13" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
     </row>
     <row r="19" spans="2:8" x14ac:dyDescent="0.25">
@@ -16701,10 +16874,10 @@
         <v>170</v>
       </c>
       <c r="C24" s="12" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="D24" s="12" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="E24" s="12" t="s">
         <v>204</v>
@@ -17353,7 +17526,7 @@
   <sheetData>
     <row r="1" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
     </row>
     <row r="2" spans="2:7" x14ac:dyDescent="0.25">
@@ -17368,7 +17541,7 @@
     </row>
     <row r="4" spans="2:7" ht="104.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="32" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="C4" s="32"/>
       <c r="D4" s="32"/>
@@ -17597,7 +17770,7 @@
         <v>240</v>
       </c>
       <c r="E17" s="27" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="F17" s="13" t="s">
         <v>87</v>
@@ -17632,7 +17805,7 @@
         <v>12</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="D19" s="13" t="s">
         <v>246</v>
@@ -17774,7 +17947,7 @@
         <v>246.62640532433457</v>
       </c>
       <c r="G28" s="27" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
     </row>
     <row r="29" spans="2:7" x14ac:dyDescent="0.25">
@@ -17792,7 +17965,7 @@
         <v>250.34991743084035</v>
       </c>
       <c r="G29" s="27" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
     </row>
   </sheetData>
@@ -17853,12 +18026,12 @@
   <sheetData>
     <row r="1" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
     </row>
     <row r="2" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B2" s="2" t="s">
-        <v>264</v>
+        <v>474</v>
       </c>
     </row>
     <row r="3" spans="2:7" x14ac:dyDescent="0.25">
@@ -17868,7 +18041,7 @@
     </row>
     <row r="4" spans="2:7" ht="225.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="32" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="C4" s="32"/>
       <c r="D4" s="32"/>
@@ -17958,14 +18131,14 @@
         <v>3</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>267</v>
+        <v>476</v>
       </c>
       <c r="D11" s="13" t="s">
         <v>233</v>
       </c>
       <c r="E11" s="6">
         <f>p_verfl</f>
-        <v>80.0</v>
+        <v>90.0</v>
       </c>
       <c r="F11" s="13" t="s">
         <v>40</v>
@@ -18026,7 +18199,7 @@
         <v>273</v>
       </c>
       <c r="E14" s="17">
-        <v>510.118773673337</v>
+        <v>516.9215185149139</v>
       </c>
       <c r="F14" s="13" t="s">
         <v>128</v>
@@ -18047,7 +18220,7 @@
       </c>
       <c r="E15" s="24">
         <f>Szen2_h1+(Szen2_h1s-Szen2_h1)/eta_V1</f>
-        <v>519.640749603479</v>
+        <v>527.739255367261</v>
       </c>
       <c r="F15" s="13" t="s">
         <v>128</v>
@@ -18067,7 +18240,7 @@
         <v>277</v>
       </c>
       <c r="E16" s="5">
-        <v>100.34728038711897</v>
+        <v>111.64303153577754</v>
       </c>
       <c r="F16" s="13" t="s">
         <v>44</v>
@@ -18109,7 +18282,7 @@
       </c>
       <c r="E18" s="21">
         <f>Szen2_h1a-Szen2_h1</f>
-        <v>59.5123495633886</v>
+        <v>67.6108553271706</v>
       </c>
       <c r="F18" s="13" t="s">
         <v>128</v>
@@ -18120,7 +18293,7 @@
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B19" s="30" t="s">
-        <v>282</v>
+        <v>475</v>
       </c>
       <c r="C19" s="30"/>
       <c r="D19" s="30"/>
@@ -18133,13 +18306,13 @@
         <v>11</v>
       </c>
       <c r="C20" s="13" t="s">
-        <v>472</v>
+        <v>477</v>
       </c>
       <c r="D20" s="13" t="s">
-        <v>473</v>
+        <v>478</v>
       </c>
       <c r="E20" s="5">
-        <v>76.65085109900227</v>
+        <v>82.17759431791859</v>
       </c>
       <c r="F20" s="13" t="s">
         <v>40</v>
@@ -18153,14 +18326,14 @@
         <v>12</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>474</v>
+        <v>479</v>
       </c>
       <c r="D21" s="13" t="s">
-        <v>475</v>
+        <v>480</v>
       </c>
       <c r="E21" s="6">
         <f>p_verfl-Szen2_psatK</f>
-        <v>3.34914890099773</v>
+        <v>7.82240568208141</v>
       </c>
       <c r="F21" s="13" t="s">
         <v>40</v>
@@ -18174,13 +18347,13 @@
         <v>13</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>476</v>
+        <v>481</v>
       </c>
       <c r="D22" s="13" t="s">
-        <v>477</v>
+        <v>482</v>
       </c>
       <c r="E22" s="5">
-        <v>23.680288076354813</v>
+        <v>76.65085109900227</v>
       </c>
       <c r="F22" s="13" t="s">
         <v>44</v>
@@ -18194,13 +18367,13 @@
         <v>14</v>
       </c>
       <c r="C23" s="13" t="s">
-        <v>289</v>
+        <v>483</v>
       </c>
       <c r="D23" s="13" t="s">
         <v>290</v>
       </c>
       <c r="E23" s="17">
-        <v>269.3649559167285</v>
+        <v>263.1108198972053</v>
       </c>
       <c r="F23" s="13" t="s">
         <v>128</v>
@@ -18214,13 +18387,13 @@
         <v>15</v>
       </c>
       <c r="C24" s="13" t="s">
-        <v>291</v>
+        <v>484</v>
       </c>
       <c r="D24" s="13" t="s">
         <v>292</v>
       </c>
       <c r="E24" s="27" t="s">
-        <v>478</v>
+        <v>485</v>
       </c>
       <c r="F24" s="13" t="s">
         <v>87</v>
@@ -18229,7 +18402,7 @@
         <v>224</v>
       </c>
       <c r="I24" s="25" t="s">
-        <v>479</v>
+        <v>487</v>
       </c>
     </row>
     <row r="25" spans="2:9" x14ac:dyDescent="0.25">
@@ -18244,7 +18417,7 @@
       </c>
       <c r="E25" s="24">
         <f>Szen2_h1a-Szen2_hV</f>
-        <v>250.275793686751</v>
+        <v>264.628435470056</v>
       </c>
       <c r="F25" s="13" t="s">
         <v>128</v>
@@ -18295,7 +18468,7 @@
         <v>299</v>
       </c>
       <c r="E28" s="17">
-        <v>274.19282277342074</v>
+        <v>266.42357229030523</v>
       </c>
       <c r="F28" s="13" t="s">
         <v>128</v>
@@ -18316,7 +18489,7 @@
       </c>
       <c r="E29" s="24">
         <f>Szen2_hV+(Szen2_hPs-Szen2_hV)/eta</f>
-        <v>275.399789487594</v>
+        <v>267.25176038858</v>
       </c>
       <c r="F29" s="13" t="s">
         <v>128</v>
@@ -18336,7 +18509,7 @@
         <v>301</v>
       </c>
       <c r="E30" s="17">
-        <v>26.993208266177675</v>
+        <v>24.35642319690257</v>
       </c>
       <c r="F30" s="13" t="s">
         <v>44</v>
@@ -18357,7 +18530,7 @@
       </c>
       <c r="E31" s="21">
         <f>Szen2_hPa-Szen2_hV</f>
-        <v>6.03483357086532</v>
+        <v>4.14094049137492</v>
       </c>
       <c r="F31" s="13" t="s">
         <v>128</v>
@@ -18388,7 +18561,7 @@
       </c>
       <c r="E33" s="21">
         <f>Szen2_w1+Szen2_wP</f>
-        <v>65.5471831342539</v>
+        <v>71.7517958185455</v>
       </c>
       <c r="F33" s="13" t="s">
         <v>128</v>
@@ -18409,7 +18582,7 @@
       </c>
       <c r="E34" s="22">
         <f>Szen1_mmin*Szen2_w_ges</f>
-        <v>1760.92962532471</v>
+        <v>1927.61697582543</v>
       </c>
       <c r="F34" s="13" t="s">
         <v>131</v>
@@ -18430,7 +18603,7 @@
       </c>
       <c r="E35" s="22">
         <f>Szen1_mmax*Szen2_w_ges</f>
-        <v>3521.85925064942</v>
+        <v>3855.23395165087</v>
       </c>
       <c r="F35" s="13" t="s">
         <v>131</v>
@@ -18444,14 +18617,14 @@
         <v>25</v>
       </c>
       <c r="C36" s="13" t="s">
-        <v>311</v>
+        <v>486</v>
       </c>
       <c r="D36" s="13" t="s">
         <v>312</v>
       </c>
       <c r="E36" s="22">
         <f>Szen1_mmax*Szen2_qV</f>
-        <v>13447.3531441305</v>
+        <v>14218.5225799285</v>
       </c>
       <c r="F36" s="13" t="s">
         <v>131</v>
@@ -18467,7 +18640,7 @@
     </row>
     <row r="39" spans="2:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B39" s="31" t="s">
-        <v>314</v>
+        <v>489</v>
       </c>
       <c r="C39" s="31"/>
       <c r="D39" s="31"/>
@@ -18477,7 +18650,7 @@
     </row>
     <row r="40" spans="2:7" ht="36.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B40" s="32" t="s">
-        <v>480</v>
+        <v>488</v>
       </c>
       <c r="C40" s="32"/>
       <c r="D40" s="32"/>
@@ -18527,7 +18700,7 @@
       </c>
       <c r="E43" s="6">
         <f>SQRT(p_S2*p_verfl)</f>
-        <v>48.9897948556636</v>
+        <v>51.9615242270663</v>
       </c>
       <c r="F43" s="13" t="s">
         <v>40</v>
@@ -18568,7 +18741,7 @@
         <v>321</v>
       </c>
       <c r="E45" s="17">
-        <v>483.7488120724261</v>
+        <v>486.7613752582456</v>
       </c>
       <c r="F45" s="13" t="s">
         <v>128</v>
@@ -18589,7 +18762,7 @@
       </c>
       <c r="E46" s="24">
         <f>Szen2_h1+(Szen2v_h1s-Szen2_h1)/eta_V1</f>
-        <v>488.247938173823</v>
+        <v>491.834322918847</v>
       </c>
       <c r="F46" s="13" t="s">
         <v>128</v>
@@ -18609,7 +18782,7 @@
         <v>322</v>
       </c>
       <c r="E47" s="5">
-        <v>55.72047810494509</v>
+        <v>60.87327000646022</v>
       </c>
       <c r="F47" s="13" t="s">
         <v>44</v>
@@ -18630,7 +18803,7 @@
       </c>
       <c r="E48" s="21">
         <f>Szen2v_h1a-Szen2_h1</f>
-        <v>28.1195381337328</v>
+        <v>31.705922878756</v>
       </c>
       <c r="F48" s="13" t="s">
         <v>128</v>
@@ -18660,7 +18833,7 @@
         <v>327</v>
       </c>
       <c r="E50" s="17">
-        <v>436.78233782651</v>
+        <v>430.8017410524622</v>
       </c>
       <c r="F50" s="13" t="s">
         <v>128</v>
@@ -18681,7 +18854,7 @@
       </c>
       <c r="E51" s="24">
         <f>Szen2v_h1a-Szen2v_hZK</f>
-        <v>51.4656003473133</v>
+        <v>61.0325818663844</v>
       </c>
       <c r="F51" s="13" t="s">
         <v>128</v>
@@ -18732,7 +18905,7 @@
         <v>330</v>
       </c>
       <c r="E54" s="17">
-        <v>457.1138194731295</v>
+        <v>452.8792553404791</v>
       </c>
       <c r="F54" s="13" t="s">
         <v>128</v>
@@ -18753,7 +18926,7 @@
       </c>
       <c r="E55" s="24">
         <f>Szen2v_hZK+(Szen2v_h2s-Szen2v_hZK)/eta_V2</f>
-        <v>461.576827639461</v>
+        <v>457.725538964678</v>
       </c>
       <c r="F55" s="13" t="s">
         <v>128</v>
@@ -18773,7 +18946,7 @@
         <v>277</v>
       </c>
       <c r="E56" s="5">
-        <v>60.65498867459198</v>
+        <v>65.20295326498872</v>
       </c>
       <c r="F56" s="13" t="s">
         <v>44</v>
@@ -18794,7 +18967,7 @@
       </c>
       <c r="E57" s="21">
         <f>Szen2v_h2a-Szen2v_hZK</f>
-        <v>24.7944898129506</v>
+        <v>26.9237979122158</v>
       </c>
       <c r="F57" s="13" t="s">
         <v>128</v>
@@ -18805,7 +18978,7 @@
     </row>
     <row r="58" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B58" s="30" t="s">
-        <v>334</v>
+        <v>490</v>
       </c>
       <c r="C58" s="30"/>
       <c r="D58" s="30"/>
@@ -18818,14 +18991,14 @@
         <v>14</v>
       </c>
       <c r="C59" s="13" t="s">
-        <v>335</v>
+        <v>491</v>
       </c>
       <c r="D59" s="13" t="s">
         <v>295</v>
       </c>
       <c r="E59" s="24">
         <f>Szen2v_h2a-Szen2_hV</f>
-        <v>192.211871722732</v>
+        <v>194.614719067473</v>
       </c>
       <c r="F59" s="13" t="s">
         <v>128</v>
@@ -18846,7 +19019,7 @@
       </c>
       <c r="E60" s="24">
         <f>Szen2_wP</f>
-        <v>6.03483357086532</v>
+        <v>4.14094049137492</v>
       </c>
       <c r="F60" s="13" t="s">
         <v>128</v>
@@ -18877,7 +19050,7 @@
       </c>
       <c r="E62" s="21">
         <f>Szen2v_w1+Szen2v_w2+Szen2_wP</f>
-        <v>58.9488615175487</v>
+        <v>62.7706612823467</v>
       </c>
       <c r="F62" s="13" t="s">
         <v>128</v>
@@ -18898,7 +19071,7 @@
       </c>
       <c r="E63" s="22">
         <f>Szen1_mmax*Szen2v_w_ges</f>
-        <v>3167.33051404519</v>
+        <v>3372.6763460425</v>
       </c>
       <c r="F63" s="13" t="s">
         <v>131</v>
@@ -18919,7 +19092,7 @@
       </c>
       <c r="E64" s="28">
         <f>1-Szen2v_w_ges/Szen2_w_ges</f>
-        <v>0.100665220093295</v>
+        <v>0.125169473930819</v>
       </c>
       <c r="F64" s="13" t="s">
         <v>87</v>
@@ -18940,7 +19113,7 @@
     </row>
     <row r="68" spans="2:7" ht="63.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B68" s="32" t="s">
-        <v>481</v>
+        <v>492</v>
       </c>
       <c r="C68" s="32"/>
       <c r="D68" s="32"/>
@@ -19162,7 +19335,7 @@
         <v>343</v>
       </c>
       <c r="D80" s="13" t="s">
-        <v>482</v>
+        <v>493</v>
       </c>
       <c r="E80" s="19" t="str">
         <f>IF(p_zw&lt;=p_tau_TK-U_PG,"✔ gasförmig (≥ 3 bar unter der Taulinie)","⚠ zu nah an der Taulinie – Zwischendruck senken")</f>
@@ -19393,7 +19566,7 @@
       </c>
       <c r="E92" s="24">
         <f>Szen2_TPa</f>
-        <v>26.9932082661777</v>
+        <v>24.3564231969026</v>
       </c>
       <c r="F92" s="13" t="s">
         <v>44</v>
@@ -19413,7 +19586,7 @@
         <v>351</v>
       </c>
       <c r="E93" s="17">
-        <v>275.39978948753435</v>
+        <v>267.2517603885796</v>
       </c>
       <c r="F93" s="13" t="s">
         <v>128</v>
@@ -19434,7 +19607,7 @@
       </c>
       <c r="E94" s="24">
         <f>Dv_h2a-Dv_hN</f>
-        <v>202.956379488294</v>
+        <v>211.104408587248</v>
       </c>
       <c r="F94" s="13" t="s">
         <v>128</v>
@@ -19486,7 +19659,7 @@
       </c>
       <c r="E97" s="21">
         <f>Dv_qZK1+Dv_qN</f>
-        <v>257.627234941271</v>
+        <v>265.775264040225</v>
       </c>
       <c r="F97" s="13" t="s">
         <v>128</v>
@@ -19530,10 +19703,10 @@
         <v>439</v>
       </c>
       <c r="E102" s="12" t="s">
-        <v>483</v>
+        <v>494</v>
       </c>
       <c r="F102" s="12" t="s">
-        <v>359</v>
+        <v>495</v>
       </c>
       <c r="G102" s="12" t="s">
         <v>360</v>
@@ -19549,11 +19722,11 @@
       </c>
       <c r="E103" s="24">
         <f>Szen2_w1</f>
-        <v>59.5123495633886</v>
+        <v>67.6108553271706</v>
       </c>
       <c r="F103" s="24">
         <f>Szen2v_w1</f>
-        <v>28.1195381337328</v>
+        <v>31.705922878756</v>
       </c>
       <c r="G103" s="24">
         <f>Dv_w1</f>
@@ -19573,7 +19746,7 @@
       </c>
       <c r="F104" s="24">
         <f>Szen2v_w2</f>
-        <v>24.7944898129506</v>
+        <v>26.9237979122158</v>
       </c>
       <c r="G104" s="24">
         <f>Dv_w2</f>
@@ -19591,11 +19764,11 @@
       </c>
       <c r="E105" s="24">
         <f>Szen2_wP</f>
-        <v>6.03483357086532</v>
+        <v>4.14094049137492</v>
       </c>
       <c r="F105" s="24">
         <f>Szen2_wP</f>
-        <v>6.03483357086532</v>
+        <v>4.14094049137492</v>
       </c>
       <c r="G105" s="24">
         <v>0</v>
@@ -19612,11 +19785,11 @@
       </c>
       <c r="E106" s="21">
         <f>SUM(E103:E105)</f>
-        <v>65.5471831342539</v>
+        <v>71.7517958185455</v>
       </c>
       <c r="F106" s="21">
         <f>SUM(F103:F105)</f>
-        <v>58.9488615175487</v>
+        <v>62.7706612823467</v>
       </c>
       <c r="G106" s="21">
         <f>SUM(G103:G105)</f>
@@ -19633,15 +19806,15 @@
       </c>
       <c r="E107" s="24">
         <f>Szen2_qV</f>
-        <v>250.275793686751</v>
+        <v>264.628435470056</v>
       </c>
       <c r="F107" s="24">
         <f>Szen2v_qZK+Szen2v_qV</f>
-        <v>243.677472070046</v>
+        <v>255.647300933857</v>
       </c>
       <c r="G107" s="24">
         <f>Dv_q_ges</f>
-        <v>257.627234941271</v>
+        <v>265.775264040225</v>
       </c>
     </row>
     <row r="108" spans="2:7" x14ac:dyDescent="0.25">
@@ -19652,18 +19825,18 @@
       <c r="D108" s="13"/>
       <c r="E108" s="20">
         <f>1-E106/G106</f>
-        <v>0.100844718485505</v>
+        <v>0.0157318273120445</v>
       </c>
       <c r="F108" s="20">
         <f>1-F106/G106</f>
-        <v>0.19135838279721</v>
+        <v>0.138932156694244</v>
       </c>
       <c r="G108" s="13"/>
     </row>
     <row r="109" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B109" s="29" t="str">
-        <f>"Ergebnis: Verflüssigen und Pumpen (S2) braucht "&amp;TEXT(1-Szen2_w_ges/Dv_w_ges,"0%")&amp;" weniger Arbeit als Durchverdichten; eine zweite Verdichterstufe spart weitere "&amp;TEXT(1-Szen2v_w_ges/Szen2_w_ges,"0%")&amp;"."</f>
-        <v>Ergebnis: Verflüssigen und Pumpen (S2) braucht 10% weniger Arbeit als Durchverdichten; eine zweite Verdichterstufe spart weitere 10%.</v>
+        <f>"Ergebnis: Die zweite Verdichterstufe ist beim Gemisch Pflicht (1 Stufe &gt; 95 °C) und spart "&amp;TEXT(1-Szen2v_w_ges/Szen2_w_ges,"0%")&amp;" gegenüber einer Stufe. Dicht kühlen und pumpen (2 Stufen) braucht "&amp;TEXT(1-Szen2v_w_ges/Dv_w_ges,"0%")&amp;" weniger Arbeit als Durchverdichten."</f>
+        <v>Ergebnis: Die zweite Verdichterstufe ist beim Gemisch Pflicht (1 Stufe &gt; 95 °C) und spart 13% gegenüber einer Stufe. Dicht kühlen und pumpen (2 Stufen) braucht 14% weniger Arbeit als Durchverdichten.</v>
       </c>
     </row>
   </sheetData>
@@ -19802,12 +19975,12 @@
   <sheetData>
     <row r="1" spans="2:2" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
-        <v>484</v>
+        <v>496</v>
       </c>
     </row>
     <row r="2" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B2" s="2" t="s">
-        <v>485</v>
+        <v>497</v>
       </c>
     </row>
     <row r="3" spans="2:2" x14ac:dyDescent="0.25">
@@ -19822,7 +19995,7 @@
     </row>
     <row r="36" spans="2:17" ht="50.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B36" s="32" t="s">
-        <v>486</v>
+        <v>498</v>
       </c>
       <c r="C36" s="32"/>
       <c r="D36" s="32"/>
@@ -19867,7 +20040,7 @@
     </row>
     <row r="72" spans="2:17" ht="158.44999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B72" s="32" t="s">
-        <v>487</v>
+        <v>499</v>
       </c>
       <c r="C72" s="32"/>
       <c r="D72" s="32"/>
@@ -20064,46 +20237,46 @@
     </row>
     <row r="16">
       <c r="B16" s="10" t="s">
-        <v>488</v>
+        <v>500</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>489</v>
+        <v>501</v>
       </c>
       <c r="D16" s="13" t="s">
-        <v>490</v>
+        <v>502</v>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="10" t="s">
-        <v>491</v>
+        <v>503</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>492</v>
+        <v>504</v>
       </c>
       <c r="D17" s="13" t="s">
-        <v>493</v>
+        <v>505</v>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="10" t="s">
-        <v>494</v>
+        <v>506</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>495</v>
+        <v>507</v>
       </c>
       <c r="D18" s="13" t="s">
-        <v>496</v>
+        <v>508</v>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="10" t="s">
-        <v>497</v>
+        <v>509</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>498</v>
+        <v>510</v>
       </c>
       <c r="D19" s="13" t="s">
-        <v>499</v>
+        <v>511</v>
       </c>
     </row>
   </sheetData>
@@ -20121,7 +20294,7 @@
     <tabColor rgb="FFD9D9D9"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:L388"/>
+  <dimension ref="B1:L408"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.7109375" customWidth="1"/>
@@ -20138,7 +20311,7 @@
     </row>
     <row r="2" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2" s="2" t="s">
-        <v>500</v>
+        <v>512</v>
       </c>
     </row>
     <row r="3" spans="2:12" x14ac:dyDescent="0.25">
@@ -20192,7 +20365,7 @@
         <v>374</v>
       </c>
       <c r="H7" s="12" t="s">
-        <v>501</v>
+        <v>513</v>
       </c>
       <c r="I7" s="12" t="s">
         <v>375</v>
@@ -20231,7 +20404,7 @@
         <v>0.0</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>502</v>
+        <v>514</v>
       </c>
       <c r="J8">
         <v>-56.557999999999964</v>
@@ -24000,7 +24173,7 @@
         <v>28.674580252176824</v>
       </c>
       <c r="I123" s="10" t="s">
-        <v>503</v>
+        <v>515</v>
       </c>
       <c r="J123">
         <v>27.954721274532744</v>
@@ -24156,7 +24329,7 @@
         <v>27.8897123459386</v>
       </c>
       <c r="I128" s="10" t="s">
-        <v>383</v>
+        <v>516</v>
       </c>
       <c r="J128">
         <f>T_S2</f>
@@ -24195,15 +24368,15 @@
       </c>
       <c r="J129">
         <f>Szen2_T1a</f>
-        <v>100.347280387119</v>
+        <v>111.643031535778</v>
       </c>
       <c r="K129">
         <f>p_verfl</f>
-        <v>80.0</v>
+        <v>90.0</v>
       </c>
       <c r="L129">
         <f>(J129-Diagramm_Tmin)/Diagramm_dT+1</f>
-        <v>361.694560774238</v>
+        <v>384.286063071555</v>
       </c>
     </row>
     <row r="130" x14ac:dyDescent="0.25">
@@ -24234,7 +24407,7 @@
       </c>
       <c r="K130">
         <f>p_verfl</f>
-        <v>80.0</v>
+        <v>90.0</v>
       </c>
       <c r="L130">
         <f>(J130-Diagramm_Tmin)/Diagramm_dT+1</f>
@@ -24265,7 +24438,7 @@
       </c>
       <c r="J131">
         <f>Szen2_TPa</f>
-        <v>26.9932082661777</v>
+        <v>24.3564231969026</v>
       </c>
       <c r="K131">
         <f>Kopf_voll</f>
@@ -24273,7 +24446,7 @@
       </c>
       <c r="L131">
         <f>(J131-Diagramm_Tmin)/Diagramm_dT+1</f>
-        <v>214.986416532355</v>
+        <v>209.712846393805</v>
       </c>
     </row>
     <row r="132" x14ac:dyDescent="0.25">
@@ -24361,15 +24534,15 @@
       </c>
       <c r="J134">
         <f>Szen2v_T1a</f>
-        <v>55.7204781049451</v>
+        <v>60.8732700064602</v>
       </c>
       <c r="K134">
         <f>Szen2v_pzw</f>
-        <v>48.9897948556636</v>
+        <v>51.9615242270663</v>
       </c>
       <c r="L134">
         <f>(J134-Diagramm_Tmin)/Diagramm_dT+1</f>
-        <v>272.44095620989</v>
+        <v>282.74654001292</v>
       </c>
     </row>
     <row r="135" x14ac:dyDescent="0.25">
@@ -24400,7 +24573,7 @@
       </c>
       <c r="K135">
         <f>Szen2v_pzw</f>
-        <v>48.9897948556636</v>
+        <v>51.9615242270663</v>
       </c>
       <c r="L135">
         <f>(J135-Diagramm_Tmin)/Diagramm_dT+1</f>
@@ -24431,15 +24604,15 @@
       </c>
       <c r="J136">
         <f>Szen2v_T2a</f>
-        <v>60.654988674592</v>
+        <v>65.2029532649887</v>
       </c>
       <c r="K136">
         <f>p_verfl</f>
-        <v>80.0</v>
+        <v>90.0</v>
       </c>
       <c r="L136">
         <f>(J136-Diagramm_Tmin)/Diagramm_dT+1</f>
-        <v>282.309977349184</v>
+        <v>291.405906529977</v>
       </c>
     </row>
     <row r="137" x14ac:dyDescent="0.25">
@@ -24632,7 +24805,7 @@
       </c>
       <c r="J142">
         <f>Szen2_TPa</f>
-        <v>26.9932082661777</v>
+        <v>24.3564231969026</v>
       </c>
       <c r="K142">
         <f>Kopf_voll</f>
@@ -24640,7 +24813,7 @@
       </c>
       <c r="L142">
         <f>(J142-Diagramm_Tmin)/Diagramm_dT+1</f>
-        <v>214.986416532355</v>
+        <v>209.712846393805</v>
       </c>
     </row>
     <row r="143" x14ac:dyDescent="0.25">
@@ -24926,14 +25099,14 @@
         <v>24.484057818450818</v>
       </c>
       <c r="J151">
-        <v>92.34728038711897</v>
+        <v>99.64303153577754</v>
       </c>
       <c r="K151">
-        <v>85.0</v>
+        <v>95.0</v>
       </c>
       <c r="L151">
         <f t="shared" si="8"/>
-        <v>345.694560774238</v>
+        <v>360.286063071555</v>
       </c>
     </row>
     <row r="152" x14ac:dyDescent="0.25">
@@ -24959,14 +25132,14 @@
         <v>24.339976664075426</v>
       </c>
       <c r="J152">
-        <v>8.0</v>
+        <v>45.0</v>
       </c>
       <c r="K152">
-        <v>80.0</v>
+        <v>94.0</v>
       </c>
       <c r="L152">
         <f t="shared" si="8"/>
-        <v>177.0</v>
+        <v>251.0</v>
       </c>
     </row>
     <row r="153" x14ac:dyDescent="0.25">
@@ -26049,7 +26222,7 @@
         <v>19.236856999637254</v>
       </c>
       <c r="I184" s="10" t="s">
-        <v>504</v>
+        <v>517</v>
       </c>
       <c r="J184">
         <f>'Kaverne &amp; Gassäule'!$C$49</f>
@@ -27948,7 +28121,7 @@
         <v>0.0</v>
       </c>
       <c r="I239" s="10" t="s">
-        <v>505</v>
+        <v>518</v>
       </c>
       <c r="J239">
         <f>Tober_V1</f>
@@ -28493,7 +28666,7 @@
         <v>0.0</v>
       </c>
       <c r="I256" s="10" t="s">
-        <v>506</v>
+        <v>519</v>
       </c>
       <c r="J256">
         <v>-56.557999999999964</v>
@@ -29873,7 +30046,7 @@
         <v>0.0</v>
       </c>
       <c r="I298" s="10" t="s">
-        <v>507</v>
+        <v>520</v>
       </c>
       <c r="J298">
         <v>-56.557999999999964</v>
@@ -30890,7 +31063,7 @@
         <v>0.0</v>
       </c>
       <c r="I329" s="10" t="s">
-        <v>508</v>
+        <v>521</v>
       </c>
       <c r="J329">
         <v>-56.557999999999964</v>
@@ -31905,6 +32078,19 @@
       <c r="H360">
         <v>0.0</v>
       </c>
+      <c r="I360" s="10" t="s">
+        <v>522</v>
+      </c>
+      <c r="J360">
+        <v>15.0</v>
+      </c>
+      <c r="K360">
+        <v>30.0</v>
+      </c>
+      <c r="L360">
+        <f>(J360-Diagramm_Tmin)/Diagramm_dT+1</f>
+        <v>191.0</v>
+      </c>
     </row>
     <row r="361" x14ac:dyDescent="0.25">
       <c r="B361">
@@ -31928,6 +32114,16 @@
       <c r="H361">
         <v>0.0</v>
       </c>
+      <c r="J361">
+        <v>73.69576974275476</v>
+      </c>
+      <c r="K361">
+        <v>60.0</v>
+      </c>
+      <c r="L361">
+        <f>(J361-Diagramm_Tmin)/Diagramm_dT+1</f>
+        <v>308.39153948551</v>
+      </c>
     </row>
     <row r="362" x14ac:dyDescent="0.25">
       <c r="B362">
@@ -31951,6 +32147,16 @@
       <c r="H362">
         <v>0.0</v>
       </c>
+      <c r="J362">
+        <v>20.0</v>
+      </c>
+      <c r="K362">
+        <v>60.0</v>
+      </c>
+      <c r="L362">
+        <f>(J362-Diagramm_Tmin)/Diagramm_dT+1</f>
+        <v>201.0</v>
+      </c>
     </row>
     <row r="363" x14ac:dyDescent="0.25">
       <c r="B363">
@@ -32548,6 +32754,467 @@
         <v>0.0</v>
       </c>
       <c r="H388">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="389">
+      <c r="B389">
+        <v>110.5</v>
+      </c>
+      <c r="C389">
+        <f>IF(MOD(B389,20)=0,TEXT(B389,"0"),"")</f>
+      </c>
+      <c r="D389">
+        <v>81.45505572191325</v>
+      </c>
+      <c r="E389">
+        <v>0.0</v>
+      </c>
+      <c r="F389">
+        <v>168.54494427808675</v>
+      </c>
+      <c r="G389">
+        <v>0.0</v>
+      </c>
+      <c r="H389">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="390">
+      <c r="B390">
+        <v>111.0</v>
+      </c>
+      <c r="C390">
+        <f>IF(MOD(B390,20)=0,TEXT(B390,"0"),"")</f>
+      </c>
+      <c r="D390">
+        <v>81.45505572191325</v>
+      </c>
+      <c r="E390">
+        <v>0.0</v>
+      </c>
+      <c r="F390">
+        <v>168.54494427808675</v>
+      </c>
+      <c r="G390">
+        <v>0.0</v>
+      </c>
+      <c r="H390">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="391">
+      <c r="B391">
+        <v>111.5</v>
+      </c>
+      <c r="C391">
+        <f>IF(MOD(B391,20)=0,TEXT(B391,"0"),"")</f>
+      </c>
+      <c r="D391">
+        <v>81.45505572191325</v>
+      </c>
+      <c r="E391">
+        <v>0.0</v>
+      </c>
+      <c r="F391">
+        <v>168.54494427808675</v>
+      </c>
+      <c r="G391">
+        <v>0.0</v>
+      </c>
+      <c r="H391">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="392">
+      <c r="B392">
+        <v>112.0</v>
+      </c>
+      <c r="C392">
+        <f>IF(MOD(B392,20)=0,TEXT(B392,"0"),"")</f>
+      </c>
+      <c r="D392">
+        <v>81.45505572191325</v>
+      </c>
+      <c r="E392">
+        <v>0.0</v>
+      </c>
+      <c r="F392">
+        <v>168.54494427808675</v>
+      </c>
+      <c r="G392">
+        <v>0.0</v>
+      </c>
+      <c r="H392">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="393">
+      <c r="B393">
+        <v>112.5</v>
+      </c>
+      <c r="C393">
+        <f>IF(MOD(B393,20)=0,TEXT(B393,"0"),"")</f>
+      </c>
+      <c r="D393">
+        <v>81.45505572191325</v>
+      </c>
+      <c r="E393">
+        <v>0.0</v>
+      </c>
+      <c r="F393">
+        <v>168.54494427808675</v>
+      </c>
+      <c r="G393">
+        <v>0.0</v>
+      </c>
+      <c r="H393">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="394">
+      <c r="B394">
+        <v>113.0</v>
+      </c>
+      <c r="C394">
+        <f>IF(MOD(B394,20)=0,TEXT(B394,"0"),"")</f>
+      </c>
+      <c r="D394">
+        <v>81.45505572191325</v>
+      </c>
+      <c r="E394">
+        <v>0.0</v>
+      </c>
+      <c r="F394">
+        <v>168.54494427808675</v>
+      </c>
+      <c r="G394">
+        <v>0.0</v>
+      </c>
+      <c r="H394">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="395">
+      <c r="B395">
+        <v>113.5</v>
+      </c>
+      <c r="C395">
+        <f>IF(MOD(B395,20)=0,TEXT(B395,"0"),"")</f>
+      </c>
+      <c r="D395">
+        <v>81.45505572191325</v>
+      </c>
+      <c r="E395">
+        <v>0.0</v>
+      </c>
+      <c r="F395">
+        <v>168.54494427808675</v>
+      </c>
+      <c r="G395">
+        <v>0.0</v>
+      </c>
+      <c r="H395">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="396">
+      <c r="B396">
+        <v>114.0</v>
+      </c>
+      <c r="C396">
+        <f>IF(MOD(B396,20)=0,TEXT(B396,"0"),"")</f>
+      </c>
+      <c r="D396">
+        <v>81.45505572191325</v>
+      </c>
+      <c r="E396">
+        <v>0.0</v>
+      </c>
+      <c r="F396">
+        <v>168.54494427808675</v>
+      </c>
+      <c r="G396">
+        <v>0.0</v>
+      </c>
+      <c r="H396">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="397">
+      <c r="B397">
+        <v>114.5</v>
+      </c>
+      <c r="C397">
+        <f>IF(MOD(B397,20)=0,TEXT(B397,"0"),"")</f>
+      </c>
+      <c r="D397">
+        <v>81.45505572191325</v>
+      </c>
+      <c r="E397">
+        <v>0.0</v>
+      </c>
+      <c r="F397">
+        <v>168.54494427808675</v>
+      </c>
+      <c r="G397">
+        <v>0.0</v>
+      </c>
+      <c r="H397">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="398">
+      <c r="B398">
+        <v>115.0</v>
+      </c>
+      <c r="C398">
+        <f>IF(MOD(B398,20)=0,TEXT(B398,"0"),"")</f>
+      </c>
+      <c r="D398">
+        <v>81.45505572191325</v>
+      </c>
+      <c r="E398">
+        <v>0.0</v>
+      </c>
+      <c r="F398">
+        <v>168.54494427808675</v>
+      </c>
+      <c r="G398">
+        <v>0.0</v>
+      </c>
+      <c r="H398">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="399">
+      <c r="B399">
+        <v>115.5</v>
+      </c>
+      <c r="C399">
+        <f>IF(MOD(B399,20)=0,TEXT(B399,"0"),"")</f>
+      </c>
+      <c r="D399">
+        <v>81.45505572191325</v>
+      </c>
+      <c r="E399">
+        <v>0.0</v>
+      </c>
+      <c r="F399">
+        <v>168.54494427808675</v>
+      </c>
+      <c r="G399">
+        <v>0.0</v>
+      </c>
+      <c r="H399">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="400">
+      <c r="B400">
+        <v>116.0</v>
+      </c>
+      <c r="C400">
+        <f>IF(MOD(B400,20)=0,TEXT(B400,"0"),"")</f>
+      </c>
+      <c r="D400">
+        <v>81.45505572191325</v>
+      </c>
+      <c r="E400">
+        <v>0.0</v>
+      </c>
+      <c r="F400">
+        <v>168.54494427808675</v>
+      </c>
+      <c r="G400">
+        <v>0.0</v>
+      </c>
+      <c r="H400">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="401">
+      <c r="B401">
+        <v>116.5</v>
+      </c>
+      <c r="C401">
+        <f>IF(MOD(B401,20)=0,TEXT(B401,"0"),"")</f>
+      </c>
+      <c r="D401">
+        <v>81.45505572191325</v>
+      </c>
+      <c r="E401">
+        <v>0.0</v>
+      </c>
+      <c r="F401">
+        <v>168.54494427808675</v>
+      </c>
+      <c r="G401">
+        <v>0.0</v>
+      </c>
+      <c r="H401">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="402">
+      <c r="B402">
+        <v>117.0</v>
+      </c>
+      <c r="C402">
+        <f>IF(MOD(B402,20)=0,TEXT(B402,"0"),"")</f>
+      </c>
+      <c r="D402">
+        <v>81.45505572191325</v>
+      </c>
+      <c r="E402">
+        <v>0.0</v>
+      </c>
+      <c r="F402">
+        <v>168.54494427808675</v>
+      </c>
+      <c r="G402">
+        <v>0.0</v>
+      </c>
+      <c r="H402">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="403">
+      <c r="B403">
+        <v>117.5</v>
+      </c>
+      <c r="C403">
+        <f>IF(MOD(B403,20)=0,TEXT(B403,"0"),"")</f>
+      </c>
+      <c r="D403">
+        <v>81.45505572191325</v>
+      </c>
+      <c r="E403">
+        <v>0.0</v>
+      </c>
+      <c r="F403">
+        <v>168.54494427808675</v>
+      </c>
+      <c r="G403">
+        <v>0.0</v>
+      </c>
+      <c r="H403">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="404">
+      <c r="B404">
+        <v>118.0</v>
+      </c>
+      <c r="C404">
+        <f>IF(MOD(B404,20)=0,TEXT(B404,"0"),"")</f>
+      </c>
+      <c r="D404">
+        <v>81.45505572191325</v>
+      </c>
+      <c r="E404">
+        <v>0.0</v>
+      </c>
+      <c r="F404">
+        <v>168.54494427808675</v>
+      </c>
+      <c r="G404">
+        <v>0.0</v>
+      </c>
+      <c r="H404">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="405">
+      <c r="B405">
+        <v>118.5</v>
+      </c>
+      <c r="C405">
+        <f>IF(MOD(B405,20)=0,TEXT(B405,"0"),"")</f>
+      </c>
+      <c r="D405">
+        <v>81.45505572191325</v>
+      </c>
+      <c r="E405">
+        <v>0.0</v>
+      </c>
+      <c r="F405">
+        <v>168.54494427808675</v>
+      </c>
+      <c r="G405">
+        <v>0.0</v>
+      </c>
+      <c r="H405">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="406">
+      <c r="B406">
+        <v>119.0</v>
+      </c>
+      <c r="C406">
+        <f>IF(MOD(B406,20)=0,TEXT(B406,"0"),"")</f>
+      </c>
+      <c r="D406">
+        <v>81.45505572191325</v>
+      </c>
+      <c r="E406">
+        <v>0.0</v>
+      </c>
+      <c r="F406">
+        <v>168.54494427808675</v>
+      </c>
+      <c r="G406">
+        <v>0.0</v>
+      </c>
+      <c r="H406">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="407">
+      <c r="B407">
+        <v>119.5</v>
+      </c>
+      <c r="C407">
+        <f>IF(MOD(B407,20)=0,TEXT(B407,"0"),"")</f>
+      </c>
+      <c r="D407">
+        <v>81.45505572191325</v>
+      </c>
+      <c r="E407">
+        <v>0.0</v>
+      </c>
+      <c r="F407">
+        <v>168.54494427808675</v>
+      </c>
+      <c r="G407">
+        <v>0.0</v>
+      </c>
+      <c r="H407">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="408">
+      <c r="B408">
+        <v>120.0</v>
+      </c>
+      <c r="C408" t="str">
+        <f>IF(MOD(B408,20)=0,TEXT(B408,"0"),"")</f>
+        <v>120</v>
+      </c>
+      <c r="D408">
+        <v>81.45505572191325</v>
+      </c>
+      <c r="E408">
+        <v>0.0</v>
+      </c>
+      <c r="F408">
+        <v>168.54494427808675</v>
+      </c>
+      <c r="G408">
+        <v>0.0</v>
+      </c>
+      <c r="H408">
         <v>0.0</v>
       </c>
     </row>
@@ -32569,7 +33236,7 @@
     <tabColor rgb="FFCA220E"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:J45"/>
+  <dimension ref="B1:J55"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="2.7109375" customWidth="1"/>
@@ -32583,75 +33250,75 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="B1" s="1" t="s">
-        <v>509</v>
+        <v>523</v>
       </c>
     </row>
     <row r="2">
       <c r="B2" s="2" t="s">
-        <v>510</v>
+        <v>524</v>
       </c>
     </row>
     <row r="3">
       <c r="B3" s="34" t="s">
-        <v>511</v>
+        <v>525</v>
       </c>
     </row>
     <row r="5">
       <c r="B5" s="39" t="s">
-        <v>512</v>
+        <v>526</v>
       </c>
     </row>
     <row r="6" ht="48" customHeight="1">
       <c r="B6" s="35" t="s">
-        <v>513</v>
+        <v>527</v>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="39" t="s">
-        <v>514</v>
+        <v>528</v>
       </c>
       <c r="F8" s="39" t="s">
-        <v>532</v>
+        <v>546</v>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="37" t="s">
-        <v>515</v>
+        <v>529</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>516</v>
+        <v>530</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>517</v>
+        <v>531</v>
       </c>
       <c r="F9" s="37" t="s">
-        <v>533</v>
+        <v>547</v>
       </c>
       <c r="G9" s="12" t="s">
-        <v>534</v>
+        <v>548</v>
       </c>
       <c r="H9" s="12" t="s">
-        <v>535</v>
+        <v>549</v>
       </c>
       <c r="I9" s="12" t="s">
-        <v>536</v>
+        <v>550</v>
       </c>
       <c r="J9" s="12" t="s">
-        <v>537</v>
+        <v>551</v>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="33" t="s">
-        <v>518</v>
+        <v>532</v>
       </c>
       <c r="C10" s="4">
         <v>95.0</v>
       </c>
       <c r="D10" s="33" t="s">
-        <v>519</v>
+        <v>533</v>
       </c>
       <c r="F10" s="33" t="s">
-        <v>538</v>
+        <v>552</v>
       </c>
       <c r="G10" s="5">
         <v>27.954721274532744</v>
@@ -32660,24 +33327,24 @@
         <v>81.45505572191325</v>
       </c>
       <c r="I10" s="13" t="s">
-        <v>539</v>
+        <v>553</v>
       </c>
       <c r="J10" s="33" t="s">
-        <v>540</v>
+        <v>554</v>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="33" t="s">
-        <v>520</v>
+        <v>534</v>
       </c>
       <c r="C11" s="4">
         <v>2.4</v>
       </c>
       <c r="D11" s="33" t="s">
-        <v>521</v>
+        <v>535</v>
       </c>
       <c r="F11" s="33" t="s">
-        <v>541</v>
+        <v>555</v>
       </c>
       <c r="G11" s="5">
         <v>27.21311799338457</v>
@@ -32686,24 +33353,24 @@
         <v>82.17759431791859</v>
       </c>
       <c r="I11" s="13" t="s">
-        <v>542</v>
+        <v>556</v>
       </c>
       <c r="J11" s="33" t="s">
-        <v>543</v>
+        <v>557</v>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="33" t="s">
-        <v>522</v>
+        <v>536</v>
       </c>
       <c r="C12" s="4">
         <v>1.0</v>
       </c>
       <c r="D12" s="33" t="s">
-        <v>523</v>
+        <v>537</v>
       </c>
       <c r="F12" s="33" t="s">
-        <v>544</v>
+        <v>558</v>
       </c>
       <c r="G12" s="5">
         <v>28.093324350116518</v>
@@ -32712,58 +33379,58 @@
         <v>80.8964737626687</v>
       </c>
       <c r="I12" s="13" t="s">
-        <v>545</v>
+        <v>559</v>
       </c>
       <c r="J12" s="33" t="s">
-        <v>546</v>
+        <v>560</v>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="33" t="s">
-        <v>524</v>
+        <v>538</v>
       </c>
       <c r="C13" s="4">
         <v>1.0</v>
       </c>
       <c r="D13" s="33" t="s">
-        <v>525</v>
+        <v>539</v>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="33" t="s">
-        <v>526</v>
+        <v>540</v>
       </c>
       <c r="C14" s="4">
         <v>0.5</v>
       </c>
       <c r="D14" s="33" t="s">
-        <v>527</v>
+        <v>541</v>
       </c>
       <c r="F14" s="33" t="s">
-        <v>547</v>
+        <v>561</v>
       </c>
       <c r="H14" s="4">
         <v>3.0</v>
       </c>
       <c r="I14" s="13" t="s">
-        <v>548</v>
+        <v>562</v>
       </c>
       <c r="J14" s="33" t="s">
-        <v>549</v>
+        <v>563</v>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="33" t="s">
-        <v>528</v>
+        <v>542</v>
       </c>
       <c r="C15" s="4">
         <v>0.1</v>
       </c>
       <c r="D15" s="33" t="s">
-        <v>529</v>
+        <v>543</v>
       </c>
       <c r="F15" s="33" t="s">
-        <v>550</v>
+        <v>564</v>
       </c>
       <c r="G15" s="5">
         <v>20.0</v>
@@ -32772,25 +33439,25 @@
         <v>76.65085109900227</v>
       </c>
       <c r="I15" s="13" t="s">
-        <v>551</v>
+        <v>565</v>
       </c>
       <c r="J15" s="33" t="s">
-        <v>552</v>
+        <v>566</v>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="33" t="s">
-        <v>530</v>
+        <v>544</v>
       </c>
       <c r="C16" s="6">
         <f>SUM(C11:C15)</f>
         <v>5.0</v>
       </c>
       <c r="D16" s="33" t="s">
-        <v>531</v>
+        <v>545</v>
       </c>
       <c r="F16" s="33" t="s">
-        <v>553</v>
+        <v>567</v>
       </c>
       <c r="G16" s="5">
         <v>20.0</v>
@@ -32799,35 +33466,35 @@
         <v>63.37008769484278</v>
       </c>
       <c r="I16" s="13" t="s">
-        <v>554</v>
+        <v>568</v>
       </c>
       <c r="J16" s="33" t="s">
-        <v>555</v>
+        <v>569</v>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="39" t="s">
-        <v>556</v>
+        <v>570</v>
       </c>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="B19" s="37" t="s">
-        <v>557</v>
+        <v>571</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>558</v>
+        <v>572</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>559</v>
+        <v>573</v>
       </c>
       <c r="E19" s="12" t="s">
-        <v>560</v>
+        <v>574</v>
       </c>
       <c r="F19" s="12" t="s">
-        <v>561</v>
+        <v>575</v>
       </c>
       <c r="G19" s="12" t="s">
-        <v>562</v>
+        <v>576</v>
       </c>
     </row>
     <row r="20">
@@ -33096,190 +33763,316 @@
     </row>
     <row r="32">
       <c r="B32" s="36" t="s">
-        <v>563</v>
+        <v>577</v>
       </c>
     </row>
     <row r="34">
       <c r="B34" s="39" t="s">
-        <v>564</v>
+        <v>578</v>
       </c>
     </row>
     <row r="35" ht="30" customHeight="1">
       <c r="B35" s="37" t="s">
-        <v>565</v>
+        <v>579</v>
       </c>
       <c r="C35" s="12"/>
       <c r="D35" s="12" t="s">
-        <v>566</v>
+        <v>580</v>
       </c>
       <c r="E35" s="12" t="s">
-        <v>567</v>
+        <v>581</v>
       </c>
       <c r="F35" s="12" t="s">
-        <v>568</v>
+        <v>582</v>
       </c>
       <c r="G35" s="12" t="s">
-        <v>569</v>
+        <v>583</v>
       </c>
     </row>
     <row r="36" ht="30" customHeight="1">
       <c r="B36" s="33" t="s">
-        <v>570</v>
+        <v>584</v>
       </c>
       <c r="D36" s="13" t="s">
-        <v>571</v>
+        <v>585</v>
       </c>
       <c r="E36" s="13" t="s">
-        <v>572</v>
+        <v>586</v>
       </c>
       <c r="F36" s="33" t="s">
-        <v>573</v>
+        <v>587</v>
       </c>
       <c r="G36" s="33" t="s">
-        <v>574</v>
+        <v>588</v>
       </c>
     </row>
     <row r="37" ht="30" customHeight="1">
       <c r="B37" s="33" t="s">
-        <v>575</v>
+        <v>589</v>
       </c>
       <c r="D37" s="13" t="s">
-        <v>576</v>
+        <v>590</v>
       </c>
       <c r="E37" s="13" t="s">
-        <v>577</v>
+        <v>591</v>
       </c>
       <c r="F37" s="33" t="s">
-        <v>578</v>
+        <v>592</v>
       </c>
       <c r="G37" s="33" t="s">
-        <v>579</v>
+        <v>593</v>
       </c>
     </row>
     <row r="38" ht="30" customHeight="1">
       <c r="B38" s="33" t="s">
-        <v>580</v>
+        <v>594</v>
       </c>
       <c r="D38" s="13" t="s">
-        <v>581</v>
+        <v>595</v>
       </c>
       <c r="E38" s="13" t="s">
-        <v>582</v>
+        <v>596</v>
       </c>
       <c r="F38" s="33" t="s">
-        <v>583</v>
+        <v>597</v>
       </c>
       <c r="G38" s="33" t="s">
-        <v>584</v>
+        <v>598</v>
       </c>
     </row>
     <row r="39" ht="30" customHeight="1">
       <c r="B39" s="33" t="s">
-        <v>585</v>
+        <v>599</v>
       </c>
       <c r="D39" s="13" t="s">
-        <v>586</v>
+        <v>600</v>
       </c>
       <c r="E39" s="13" t="s">
-        <v>587</v>
+        <v>601</v>
       </c>
       <c r="F39" s="33" t="s">
-        <v>588</v>
+        <v>602</v>
       </c>
       <c r="G39" s="33" t="s">
-        <v>589</v>
+        <v>603</v>
       </c>
     </row>
     <row r="40" ht="30" customHeight="1">
       <c r="B40" s="33" t="s">
-        <v>590</v>
+        <v>604</v>
       </c>
       <c r="D40" s="13" t="s">
-        <v>591</v>
+        <v>605</v>
       </c>
       <c r="E40" s="13" t="s">
-        <v>592</v>
+        <v>606</v>
       </c>
       <c r="F40" s="33" t="s">
-        <v>593</v>
+        <v>607</v>
       </c>
       <c r="G40" s="33" t="s">
-        <v>594</v>
+        <v>608</v>
       </c>
     </row>
     <row r="41" ht="30" customHeight="1">
       <c r="B41" s="33" t="s">
-        <v>595</v>
+        <v>609</v>
       </c>
       <c r="D41" s="13" t="s">
-        <v>596</v>
+        <v>610</v>
       </c>
       <c r="E41" s="13" t="s">
-        <v>597</v>
+        <v>611</v>
       </c>
       <c r="F41" s="33" t="s">
-        <v>598</v>
+        <v>612</v>
       </c>
       <c r="G41" s="33" t="s">
-        <v>599</v>
+        <v>613</v>
       </c>
     </row>
     <row r="42" ht="30" customHeight="1">
       <c r="B42" s="33" t="s">
-        <v>600</v>
+        <v>614</v>
       </c>
       <c r="D42" s="13" t="s">
-        <v>601</v>
+        <v>615</v>
       </c>
       <c r="E42" s="13" t="s">
-        <v>602</v>
+        <v>616</v>
       </c>
       <c r="F42" s="33" t="s">
-        <v>603</v>
+        <v>617</v>
       </c>
       <c r="G42" s="33" t="s">
-        <v>604</v>
+        <v>618</v>
       </c>
     </row>
     <row r="43" ht="30" customHeight="1">
       <c r="B43" s="33" t="s">
-        <v>605</v>
+        <v>619</v>
       </c>
       <c r="D43" s="13" t="s">
-        <v>606</v>
+        <v>620</v>
       </c>
       <c r="E43" s="13" t="s">
-        <v>607</v>
+        <v>621</v>
       </c>
       <c r="F43" s="33" t="s">
-        <v>608</v>
+        <v>622</v>
       </c>
       <c r="G43" s="33" t="s">
-        <v>609</v>
+        <v>623</v>
       </c>
     </row>
     <row r="44" ht="30" customHeight="1">
       <c r="B44" s="33" t="s">
-        <v>610</v>
+        <v>624</v>
       </c>
       <c r="D44" s="13" t="s">
-        <v>611</v>
+        <v>625</v>
       </c>
       <c r="E44" s="13" t="s">
-        <v>612</v>
+        <v>626</v>
       </c>
       <c r="F44" s="33" t="s">
-        <v>613</v>
+        <v>627</v>
       </c>
       <c r="G44" s="33" t="s">
-        <v>614</v>
+        <v>628</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" s="39" t="s">
+        <v>629</v>
+      </c>
+    </row>
+    <row r="47" ht="30" customHeight="1">
+      <c r="B47" s="37"/>
+      <c r="C47" s="12"/>
+      <c r="D47" s="12" t="s">
+        <v>630</v>
+      </c>
+      <c r="E47" s="12" t="s">
+        <v>631</v>
+      </c>
+      <c r="F47" s="12" t="s">
+        <v>632</v>
+      </c>
+      <c r="G47" s="12"/>
+    </row>
+    <row r="48" ht="45" customHeight="1">
+      <c r="B48" s="33" t="s">
+        <v>633</v>
+      </c>
+      <c r="D48" s="13" t="s">
+        <v>634</v>
+      </c>
+      <c r="E48" s="13" t="s">
+        <v>635</v>
+      </c>
+      <c r="F48" s="33" t="s">
+        <v>636</v>
+      </c>
+    </row>
+    <row r="49" ht="45" customHeight="1">
+      <c r="B49" s="33" t="s">
+        <v>637</v>
+      </c>
+      <c r="D49" s="13" t="s">
+        <v>638</v>
+      </c>
+      <c r="E49" s="13" t="s">
+        <v>639</v>
+      </c>
+      <c r="F49" s="33" t="s">
+        <v>640</v>
+      </c>
+    </row>
+    <row r="50" ht="45" customHeight="1">
+      <c r="B50" s="33" t="s">
+        <v>641</v>
+      </c>
+      <c r="D50" s="13" t="s">
+        <v>642</v>
+      </c>
+      <c r="E50" s="13" t="s">
+        <v>643</v>
+      </c>
+      <c r="F50" s="33" t="s">
+        <v>644</v>
+      </c>
+    </row>
+    <row r="51" ht="45" customHeight="1">
+      <c r="B51" s="33" t="s">
+        <v>645</v>
+      </c>
+      <c r="D51" s="13" t="s">
+        <v>646</v>
+      </c>
+      <c r="E51" s="13" t="s">
+        <v>647</v>
+      </c>
+      <c r="F51" s="33" t="s">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="52" ht="45" customHeight="1">
+      <c r="B52" s="33" t="s">
+        <v>649</v>
+      </c>
+      <c r="D52" s="13" t="s">
+        <v>650</v>
+      </c>
+      <c r="E52" s="13" t="s">
+        <v>651</v>
+      </c>
+      <c r="F52" s="33" t="s">
+        <v>652</v>
+      </c>
+    </row>
+    <row r="53" ht="45" customHeight="1">
+      <c r="B53" s="33" t="s">
+        <v>653</v>
+      </c>
+      <c r="D53" s="13" t="s">
+        <v>654</v>
+      </c>
+      <c r="E53" s="13" t="s">
+        <v>655</v>
+      </c>
+      <c r="F53" s="33" t="s">
+        <v>656</v>
+      </c>
+    </row>
+    <row r="54" ht="45" customHeight="1">
+      <c r="B54" s="33" t="s">
+        <v>657</v>
+      </c>
+      <c r="D54" s="13" t="s">
+        <v>658</v>
+      </c>
+      <c r="E54" s="13" t="s">
+        <v>659</v>
+      </c>
+      <c r="F54" s="33" t="s">
+        <v>660</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="12">
     <mergeCell ref="B6:J6"/>
     <mergeCell ref="B32:J32"/>
     <mergeCell ref="F14:G14"/>
+    <mergeCell ref="F47:J47"/>
+    <mergeCell ref="F48:J48"/>
+    <mergeCell ref="F49:J49"/>
+    <mergeCell ref="F50:J50"/>
+    <mergeCell ref="F51:J51"/>
+    <mergeCell ref="F52:J52"/>
+    <mergeCell ref="F53:J53"/>
+    <mergeCell ref="F54:J54"/>
+    <mergeCell ref="F55:J55"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="B3" location="'Übersicht'!A1" display="← zur Übersicht"/>

</xml_diff>